<commit_message>
Fix WhoHeroes demo UI, night flow, and defender balance
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Config_whoheroes.xlsx
+++ b/Assets/StreamingAssets/Config_whoheroes.xlsx
@@ -26218,17 +26218,17 @@
       <c r="E1005" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1005" s="48" t="s">
-        <v>57</v>
+      <c r="F1005" s="48">
+        <v>2</v>
       </c>
       <c r="G1005" s="48">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="H1005" s="48">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="I1005" s="48">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="J1005" s="48" t="s">
         <v>57</v>
@@ -26370,17 +26370,17 @@
       <c r="E1006" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1006" s="48" t="s">
-        <v>57</v>
+      <c r="F1006" s="48">
+        <v>3</v>
       </c>
       <c r="G1006" s="48">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="H1006" s="48">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="I1006" s="48">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="J1006" s="48" t="s">
         <v>57</v>
@@ -26522,17 +26522,17 @@
       <c r="E1007" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1007" s="48" t="s">
-        <v>57</v>
+      <c r="F1007" s="48">
+        <v>2</v>
       </c>
       <c r="G1007" s="48">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="H1007" s="48">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I1007" s="48">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="J1007" s="48" t="s">
         <v>57</v>
@@ -26674,17 +26674,17 @@
       <c r="E1008" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1008" s="48" t="s">
-        <v>57</v>
+      <c r="F1008" s="48">
+        <v>2</v>
       </c>
       <c r="G1008" s="48">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="H1008" s="48">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="I1008" s="48">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="J1008" s="48" t="s">
         <v>57</v>
@@ -26981,17 +26981,17 @@
       <c r="E1010" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1010" s="48" t="s">
-        <v>57</v>
+      <c r="F1010" s="48">
+        <v>3</v>
       </c>
       <c r="G1010" s="48">
-        <v>100</v>
+        <v>165</v>
       </c>
       <c r="H1010" s="48">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I1010" s="48">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J1010" s="48" t="s">
         <v>57</v>
@@ -27136,17 +27136,17 @@
       <c r="E1011" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1011" s="48" t="s">
-        <v>57</v>
+      <c r="F1011" s="48">
+        <v>3</v>
       </c>
       <c r="G1011" s="48">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="H1011" s="48">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="I1011" s="48">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="J1011" s="48" t="s">
         <v>57</v>
@@ -27288,17 +27288,17 @@
       <c r="E1012" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1012" s="48" t="s">
-        <v>57</v>
+      <c r="F1012" s="48">
+        <v>3</v>
       </c>
       <c r="G1012" s="48">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="H1012" s="48">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="I1012" s="48">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="J1012" s="48" t="s">
         <v>57</v>
@@ -27440,17 +27440,17 @@
       <c r="E1013" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1013" s="48" t="s">
-        <v>57</v>
+      <c r="F1013" s="48">
+        <v>2</v>
       </c>
       <c r="G1013" s="48">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="H1013" s="48">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I1013" s="48">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="J1013" s="48" t="s">
         <v>57</v>
@@ -27592,17 +27592,17 @@
       <c r="E1014" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1014" s="48" t="s">
-        <v>57</v>
+      <c r="F1014" s="48">
+        <v>2</v>
       </c>
       <c r="G1014" s="48">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="H1014" s="48">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I1014" s="48">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="J1014" s="48" t="s">
         <v>57</v>
@@ -27744,17 +27744,17 @@
       <c r="E1015" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1015" s="48" t="s">
-        <v>57</v>
+      <c r="F1015" s="48">
+        <v>3</v>
       </c>
       <c r="G1015" s="48">
-        <v>100</v>
+        <v>135</v>
       </c>
       <c r="H1015" s="48">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="I1015" s="48">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="J1015" s="48" t="s">
         <v>57</v>
@@ -27896,17 +27896,17 @@
       <c r="E1016" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1016" s="48" t="s">
-        <v>57</v>
+      <c r="F1016" s="48">
+        <v>2</v>
       </c>
       <c r="G1016" s="48">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="H1016" s="48">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="I1016" s="48">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J1016" s="48" t="s">
         <v>57</v>
@@ -28048,17 +28048,17 @@
       <c r="E1017" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1017" s="48" t="s">
-        <v>57</v>
+      <c r="F1017" s="48">
+        <v>2</v>
       </c>
       <c r="G1017" s="48">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="H1017" s="48">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I1017" s="48">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J1017" s="48" t="s">
         <v>57</v>
@@ -28200,17 +28200,17 @@
       <c r="E1018" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1018" s="48" t="s">
-        <v>57</v>
+      <c r="F1018" s="48">
+        <v>2</v>
       </c>
       <c r="G1018" s="48">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="H1018" s="48">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I1018" s="48">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="J1018" s="48" t="s">
         <v>57</v>
@@ -28352,17 +28352,17 @@
       <c r="E1019" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1019" s="48" t="s">
-        <v>57</v>
+      <c r="F1019" s="48">
+        <v>2</v>
       </c>
       <c r="G1019" s="48">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H1019" s="48">
         <v>10</v>
       </c>
       <c r="I1019" s="48">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="J1019" s="48" t="s">
         <v>57</v>
@@ -28504,17 +28504,17 @@
       <c r="E1020" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1020" s="48" t="s">
-        <v>57</v>
+      <c r="F1020" s="48">
+        <v>2</v>
       </c>
       <c r="G1020" s="48">
-        <v>10</v>
+        <v>85</v>
       </c>
       <c r="H1020" s="48">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="I1020" s="48">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="J1020" s="48" t="s">
         <v>57</v>
@@ -28656,17 +28656,17 @@
       <c r="E1021" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1021" s="48" t="s">
-        <v>57</v>
+      <c r="F1021" s="48">
+        <v>3</v>
       </c>
       <c r="G1021" s="48">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="H1021" s="48">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="I1021" s="48">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="J1021" s="48" t="s">
         <v>57</v>
@@ -28808,17 +28808,17 @@
       <c r="E1022" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1022" s="48" t="s">
-        <v>57</v>
+      <c r="F1022" s="48">
+        <v>3</v>
       </c>
       <c r="G1022" s="48">
-        <v>50</v>
+        <v>115</v>
       </c>
       <c r="H1022" s="48">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="I1022" s="48">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="J1022" s="48" t="s">
         <v>57</v>
@@ -28960,17 +28960,17 @@
       <c r="E1023" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1023" s="48" t="s">
-        <v>57</v>
+      <c r="F1023" s="48">
+        <v>3</v>
       </c>
       <c r="G1023" s="48">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="H1023" s="48">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="I1023" s="48">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="J1023" s="48" t="s">
         <v>57</v>
@@ -29112,17 +29112,17 @@
       <c r="E1024" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1024" s="48" t="s">
-        <v>57</v>
+      <c r="F1024" s="48">
+        <v>3</v>
       </c>
       <c r="G1024" s="48">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="H1024" s="48">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="I1024" s="48">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="J1024" s="48" t="s">
         <v>57</v>
@@ -29264,17 +29264,17 @@
       <c r="E1025" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1025" s="48" t="s">
-        <v>57</v>
+      <c r="F1025" s="48">
+        <v>3</v>
       </c>
       <c r="G1025" s="48">
-        <v>10</v>
+        <v>125</v>
       </c>
       <c r="H1025" s="48">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="I1025" s="48">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="J1025" s="48" t="s">
         <v>57</v>
@@ -29416,17 +29416,17 @@
       <c r="E1026" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1026" s="48" t="s">
-        <v>57</v>
+      <c r="F1026" s="48">
+        <v>2</v>
       </c>
       <c r="G1026" s="48">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="H1026" s="48">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I1026" s="48">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="J1026" s="48" t="s">
         <v>57</v>
@@ -29568,17 +29568,17 @@
       <c r="E1027" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1027" s="48" t="s">
-        <v>57</v>
+      <c r="F1027" s="48">
+        <v>3</v>
       </c>
       <c r="G1027" s="48">
-        <v>10</v>
+        <v>130</v>
       </c>
       <c r="H1027" s="48">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="I1027" s="48">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="J1027" s="48" t="s">
         <v>57</v>
@@ -29720,17 +29720,17 @@
       <c r="E1028" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="F1028" s="48" t="s">
-        <v>57</v>
+      <c r="F1028" s="48">
+        <v>2</v>
       </c>
       <c r="G1028" s="48">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="H1028" s="48">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="I1028" s="48">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J1028" s="48" t="s">
         <v>57</v>

</xml_diff>